<commit_message>
feat: multi-object SOQL resolution, #N/A rollback clearance, and URL-safe chunking
- Implemented dynamic URL-safe SOQL chunking and parallel fetch to eliminate HTTP 431 errors
- Added multi-object relationship field resolution (traversing lookups like BT_Project__c.Project__r)
- Fixed Bulk API 2.0 rollback logic to transmit #N/A for blank fields to properly clear Salesforce values
- Added canonical object name normalization for sitetracker__Site__c
- Improved live sitetracker file detection and UI badge display
- Comprehensive test coverage for all SOQL fetching, bulk upload, and authentication profiles
</commit_message>
<xml_diff>
--- a/data/Master_Site_Listing/input/source/Source Data for Master Site Listing.xlsx
+++ b/data/Master_Site_Listing/input/source/Source Data for Master Site Listing.xlsx
@@ -16,10 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -58,12 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,11 +451,15 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>10006</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>45983</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>10006</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2025-11-22 00:00:00</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -468,16 +468,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>PASS - Numeric PK with ISO Date &amp; Uppercase text</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>10010</v>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>45984</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>10010</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2025-11-23 00:00:00</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -486,16 +490,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>PASS - Numeric PK with ISO Date &amp; Uppercase text</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>10011</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>45985</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>10011</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2025-11-24 00:00:00</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -504,16 +512,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>PASS - Numeric PK with ISO Date &amp; Lowercase text</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>10012</v>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>45986</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>10012</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2025-11-25 00:00:00</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -522,13 +534,15 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>PASS - Numeric PK with ISO Date &amp; Proper text</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>10015</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>10015</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -542,16 +556,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL - Date Error: Nov 31 does not exist</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>10016</v>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>45986</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>10016</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2025-11-25 00:00:00</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -560,13 +578,15 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>PASS - Free text allowed in text field</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>10017</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>10017</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -580,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>FAIL - Date can't be String</t>
+          <t>FAIL - Date Error: Non-date text string</t>
         </is>
       </c>
     </row>
@@ -590,8 +610,10 @@
           <t>Invalid TM Cell ID</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
-        <v>45986</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2025-11-25 00:00:00</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -600,31 +622,35 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>FAIL - Invalid Primary Key (TM Cell ID)</t>
+          <t>FAIL - PK Error: Spaces in TM Cell ID</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>10019</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>10019</t>
+        </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>PASS - Blank row (No change detected)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>10020</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>10020</t>
+        </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>PASS - Blank row (No change detected)</t>
         </is>
       </c>
     </row>
@@ -646,7 +672,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FAIL - Invalid Leap Year (2025 has no Feb 29)</t>
+          <t>FAIL - Date Error: Non-leap year Feb 29</t>
         </is>
       </c>
     </row>
@@ -668,7 +694,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>FAIL - Invalid Month (Month 13 does not exist)</t>
+          <t>FAIL - Date Error: Invalid Month 13</t>
         </is>
       </c>
     </row>
@@ -690,29 +716,483 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>FAIL - PK Not in Sitetracker</t>
+          <t>FAIL - PK Error: Numeric PK not found in Sitetracker</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>CELL-90123</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>PASS - String PK with hyphen (CELL-90123)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SITE_45A</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>29/11/2025</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>PASS - String PK with underscore (SITE_45A)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>UKLONHUB</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>30/11/2025</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>PASS - String PK pure alphabetic (UKLONHUB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>westcell</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>15/12/2025</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>PASS - String PK lowercase (westcell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ST-North_007</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>18/12/2025</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>PASS - String PK mixed case with hyphen &amp; underscore</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>00985</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>20/12/2025</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>PASS - String PK with leading zeros preserved</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CELL-90123-TRIM  </t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>22/12/2025</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>PASS - String PK with whitespace auto-trimmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TM 1004</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>25/11/2025</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>FAIL - PK Error: Internal space in String PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CELL#99</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>25/11/2025</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>FAIL - PK Error: Special char # in String PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SITE@HQ</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>25/11/2025</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>FAIL - PK Error: Special char @ in String PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>10035/B</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>25/11/2025</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>FAIL - PK Error: Special char / in String PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TM.CELL.01</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>25/11/2025</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>FAIL - PK Error: Special char . in String PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>25/11/2025</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>FAIL - PK Error: Empty/blank Primary Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SITE_STRING_TBD</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>FAIL - Date Error: TBD string in date column</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SITE_STRING_PENDING</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>FAIL - Date Error: Pending string in date column</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SITE_STRING_INV_DAY</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>35/01/2025</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>FAIL - Date Error: Day 35 does not exist</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SITE_STRING_INV_MONTH</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>20/13/2025</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>FAIL - Date Error: Month 14 does not exist</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>GHOST-CELL-999</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>01/12/2025</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>FAIL - PK Error: String PK not in Sitetracker (Skipped)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>UNCHANGED_STRING_CELL</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>10/11/2025</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>PASS - String PK with identical Sitetracker values (Skipped)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SITE_STRING_CASE_TEST</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>01/11/2025</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>PASS - String PK with lowercase yes auto-titlecased</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SITE_STRING_BLANK_DATE</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>PASS - String PK with empty date (Safe mode ignores, Insert Nulls wipes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>10006</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>22/11/2025</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>FAIL - Duplicate Primary Key</t>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>FAIL - PK Error: Duplicate Primary Key (first occurrence was processed)</t>
         </is>
       </c>
     </row>

</xml_diff>